<commit_message>
rename type to Condition
</commit_message>
<xml_diff>
--- a/output/tables/picarro_data_averaged.xlsx
+++ b/output/tables/picarro_data_averaged.xlsx
@@ -387,7 +387,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>Condition</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -417,7 +417,7 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Order_Index_type</t>
+          <t>Order_Index_Condition</t>
         </is>
       </c>
     </row>

</xml_diff>